<commit_message>
Excel con pestañas Engorde, Madres y Tostones_Saldos
</commit_message>
<xml_diff>
--- a/MATADERO CLIENTE.xlsx
+++ b/MATADERO CLIENTE.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jaumejr\Documents\GitHub\ALBARAN\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{07F5B061-7AD9-428A-BE0E-C01BBB54A8B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{734A82F5-CBCC-44B3-9FC2-57A474642315}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{E94B9CD5-808D-4231-A830-D18B584BFBCD}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="30">
   <si>
     <t>MATADERO</t>
   </si>
@@ -102,6 +102,30 @@
   </si>
   <si>
     <t>OLOT MEATS</t>
+  </si>
+  <si>
+    <t>PRIMACARNE</t>
+  </si>
+  <si>
+    <t>BARTRA</t>
+  </si>
+  <si>
+    <t>MARCIAL</t>
+  </si>
+  <si>
+    <t>BOPEPOR</t>
+  </si>
+  <si>
+    <t>TIPO</t>
+  </si>
+  <si>
+    <t>ENGORDE</t>
+  </si>
+  <si>
+    <t>MADRES</t>
+  </si>
+  <si>
+    <t>TOSTONES_SALDOS</t>
   </si>
 </sst>
 </file>
@@ -473,159 +497,260 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DA86CD20-1585-4548-B725-7E3A781943C5}">
-  <dimension ref="A1:B19"/>
+  <dimension ref="A1:C23"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>3</v>
       </c>
       <c r="B2" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>4</v>
       </c>
       <c r="B3" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>5</v>
       </c>
       <c r="B4" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C4" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>6</v>
       </c>
       <c r="B5" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C5" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>5</v>
       </c>
       <c r="B6" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C6" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>7</v>
       </c>
       <c r="B7" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C7" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>8</v>
       </c>
       <c r="B8" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C8" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>10</v>
       </c>
       <c r="B9" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C9" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>11</v>
       </c>
       <c r="B10" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C10" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>12</v>
       </c>
       <c r="B11" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C11" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>13</v>
       </c>
       <c r="B12" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C12" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>14</v>
       </c>
       <c r="B13" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C13" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>14</v>
       </c>
       <c r="B14" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C14" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>14</v>
       </c>
       <c r="B15" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C15" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>18</v>
       </c>
       <c r="B16" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C16" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>20</v>
       </c>
       <c r="B17" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C17" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>21</v>
       </c>
       <c r="B18" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C18" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>21</v>
       </c>
       <c r="B19" t="s">
         <v>16</v>
+      </c>
+      <c r="C19" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>22</v>
+      </c>
+      <c r="B20" t="s">
+        <v>22</v>
+      </c>
+      <c r="C20" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>25</v>
+      </c>
+      <c r="B21" t="s">
+        <v>25</v>
+      </c>
+      <c r="C21" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>23</v>
+      </c>
+      <c r="B22" t="s">
+        <v>23</v>
+      </c>
+      <c r="C22" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>24</v>
+      </c>
+      <c r="B23" t="s">
+        <v>24</v>
+      </c>
+      <c r="C23" t="s">
+        <v>28</v>
       </c>
     </row>
   </sheetData>

</xml_diff>